<commit_message>
Update Booking, Notification, Doctor TestCase
</commit_message>
<xml_diff>
--- a/TestCases/Booking_TestCase.xlsx
+++ b/TestCases/Booking_TestCase.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\DoAnNganh\SpringMediCareWeb-Selenium-Testing\TestCases\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E781DED-A1BE-47F8-A119-0BEE4D9E46B4}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F65AC02F-5AC2-4526-A2DE-D206E40DBE6A}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="10056" windowHeight="6960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="12012" windowHeight="6960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="BOOKING" sheetId="5" r:id="rId1"/>
@@ -23,12 +23,21 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="80">
   <si>
     <t>TEST CASE</t>
   </si>
   <si>
     <t>Test requirement:</t>
+  </si>
+  <si>
+    <t>System Name：</t>
+  </si>
+  <si>
+    <t>SpringMediCareWeb</t>
+  </si>
+  <si>
+    <t>Module Code：</t>
   </si>
   <si>
     <t>Pass</t>
@@ -65,15 +74,6 @@
   </si>
   <si>
     <t>Note</t>
-  </si>
-  <si>
-    <t>System Name：</t>
-  </si>
-  <si>
-    <t>SpringMediCareWeb</t>
-  </si>
-  <si>
-    <t>Module Code：</t>
   </si>
   <si>
     <t>Retest Date</t>
@@ -262,10 +262,11 @@
     <t>Đặt lịch trong khoảng thời gian gần với lịch hẹn đã tồn tại</t>
   </si>
   <si>
-    <t>1: Đăng nhập bằng tài khoản bệnh nhân.
-2: Quan sát thấy bác sĩ có lịch hẹn lúc cùng ngày lúc 15:30.
-3: Nhập giờ 15:31.
-4: Nhấn nút Đặt lịch.</t>
+    <t>1: Đăng nhập bằng tài khoản bệnh nhân patient_an.
+2: Đặt lịch hẹn với bác sĩ lúc 15:30 vào ngày bác sĩ có làm.
+3: Đăng xuất và đăng nhập bằng tài khoản bệnh nhân patient_chi
+4: Đặt lịch hẹn cùng ngày nhập giờ 15:31
+5: Nhấn nút Đặt lịch</t>
   </si>
   <si>
     <t>Hệ thống không cho phép tạo lịch hẹn trong khoảng thời gian gần với lịch hẹn đã tồn tại và hiển thị thông báo thời gian khám không khả dụng.</t>
@@ -279,13 +280,37 @@
   <si>
     <t>TCBookingRetest8</t>
   </si>
+  <si>
+    <t xml:space="preserve">5. Kiểm tra quyền truy cập chức năng đặt lịch        </t>
+  </si>
+  <si>
+    <t>TC-BOOKING-009</t>
+  </si>
+  <si>
+    <t>Kiểm tra nút Đặt lịch hẹn điều hướng đúng đến bác sĩ được chọn, với người dùng chưa đăng nhập.</t>
+  </si>
+  <si>
+    <t>1: Mở trang bác sĩ.
+2: Chọn một bác sĩ, ví dụ Tran Binh.
+3: Nhấn Đặt lịch hẹn trên đúng card của bác sĩ đó.
+4: Quan sát trang được điều hướng đến.</t>
+  </si>
+  <si>
+    <t>Hệ thống điều hướng sang trang Đặt lịch hẹn khám của đúng bác sĩ đã chọn. Thông tin bác sĩ trên trang đặt lịch tương ứng với Tran Binh. Không điều hướng sang bác sĩ khác và không phát sinh lỗi.</t>
+  </si>
+  <si>
+    <t>TCBooking9_1, TCBooking9_2</t>
+  </si>
+  <si>
+    <t>Guest chưa đăng nhập vẫn truy cập được trang đặt lịch. Cần bổ sung kiểm tra xác thực trước khi cho phép truy cập chức năng đặt lịch.</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="166" formatCode="d\-m"/>
+    <numFmt numFmtId="165" formatCode="d\-m"/>
   </numFmts>
   <fonts count="10" x14ac:knownFonts="1">
     <font>
@@ -293,11 +318,6 @@
       <color rgb="FF000000"/>
       <name val="MS PGothic"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Tahoma"/>
     </font>
     <font>
       <sz val="11"/>
@@ -313,6 +333,11 @@
       <sz val="11"/>
       <color theme="1"/>
       <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Tahoma"/>
     </font>
     <font>
       <b/>
@@ -408,6 +433,15 @@
       <diagonal/>
     </border>
     <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
       <left style="thin">
         <color rgb="FF000000"/>
       </left>
@@ -420,6 +454,39 @@
       <bottom style="thin">
         <color rgb="FF000000"/>
       </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
       <diagonal/>
     </border>
     <border>
@@ -459,122 +526,86 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -819,9 +850,9 @@
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="27"/>
-      <c r="C1" s="28"/>
-      <c r="D1" s="28"/>
+      <c r="B1" s="29"/>
+      <c r="C1" s="30"/>
+      <c r="D1" s="30"/>
       <c r="E1" s="2"/>
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
@@ -848,9 +879,9 @@
     </row>
     <row r="2" spans="1:27" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A2" s="2"/>
-      <c r="B2" s="26"/>
-      <c r="C2" s="26"/>
-      <c r="D2" s="26"/>
+      <c r="B2" s="28"/>
+      <c r="C2" s="28"/>
+      <c r="D2" s="28"/>
       <c r="E2" s="2"/>
       <c r="F2" s="2"/>
       <c r="G2" s="2"/>
@@ -877,13 +908,13 @@
     </row>
     <row r="3" spans="1:27" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
-        <v>14</v>
+        <v>2</v>
       </c>
-      <c r="B3" s="29" t="s">
-        <v>15</v>
+      <c r="B3" s="31" t="s">
+        <v>3</v>
       </c>
-      <c r="C3" s="22"/>
-      <c r="D3" s="24"/>
+      <c r="C3" s="24"/>
+      <c r="D3" s="26"/>
       <c r="E3" s="2"/>
       <c r="F3" s="2"/>
       <c r="G3" s="2"/>
@@ -910,13 +941,13 @@
     </row>
     <row r="4" spans="1:27" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
-        <v>16</v>
+        <v>4</v>
       </c>
-      <c r="B4" s="30" t="s">
+      <c r="B4" s="32" t="s">
         <v>21</v>
       </c>
-      <c r="C4" s="22"/>
-      <c r="D4" s="24"/>
+      <c r="C4" s="24"/>
+      <c r="D4" s="26"/>
       <c r="E4" s="2"/>
       <c r="F4" s="2"/>
       <c r="G4" s="2"/>
@@ -945,11 +976,11 @@
       <c r="A5" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="B5" s="29" t="s">
+      <c r="B5" s="31" t="s">
         <v>22</v>
       </c>
-      <c r="C5" s="22"/>
-      <c r="D5" s="24"/>
+      <c r="C5" s="24"/>
+      <c r="D5" s="26"/>
       <c r="E5" s="2"/>
       <c r="F5" s="2"/>
       <c r="G5" s="2"/>
@@ -976,13 +1007,13 @@
     </row>
     <row r="6" spans="1:27" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="B6" s="6">
         <v>7</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D6" s="8">
         <v>0</v>
@@ -1013,16 +1044,16 @@
     </row>
     <row r="7" spans="1:27" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="B7" s="6">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C7" s="9" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="D7" s="8">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E7" s="2"/>
       <c r="F7" s="2"/>
@@ -1078,39 +1109,39 @@
       <c r="AA8" s="3"/>
     </row>
     <row r="9" spans="1:27" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A9" s="31" t="s">
-        <v>6</v>
-      </c>
-      <c r="B9" s="32" t="s">
-        <v>7</v>
-      </c>
-      <c r="C9" s="31" t="s">
-        <v>8</v>
-      </c>
-      <c r="D9" s="33" t="s">
+      <c r="A9" s="33" t="s">
         <v>9</v>
       </c>
-      <c r="E9" s="28"/>
-      <c r="F9" s="28"/>
-      <c r="G9" s="31" t="s">
+      <c r="B9" s="34" t="s">
         <v>10</v>
       </c>
-      <c r="H9" s="34" t="s">
+      <c r="C9" s="33" t="s">
         <v>11</v>
       </c>
-      <c r="I9" s="34" t="s">
+      <c r="D9" s="35" t="s">
         <v>12</v>
       </c>
-      <c r="J9" s="34" t="s">
+      <c r="E9" s="30"/>
+      <c r="F9" s="30"/>
+      <c r="G9" s="33" t="s">
         <v>13</v>
       </c>
-      <c r="K9" s="34" t="s">
+      <c r="H9" s="36" t="s">
+        <v>14</v>
+      </c>
+      <c r="I9" s="36" t="s">
+        <v>15</v>
+      </c>
+      <c r="J9" s="36" t="s">
+        <v>16</v>
+      </c>
+      <c r="K9" s="36" t="s">
         <v>17</v>
       </c>
-      <c r="L9" s="34" t="s">
+      <c r="L9" s="36" t="s">
         <v>18</v>
       </c>
-      <c r="M9" s="34" t="s">
+      <c r="M9" s="36" t="s">
         <v>19</v>
       </c>
       <c r="N9" s="3"/>
@@ -1129,19 +1160,19 @@
       <c r="AA9" s="3"/>
     </row>
     <row r="10" spans="1:27" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A10" s="23"/>
-      <c r="B10" s="23"/>
-      <c r="C10" s="23"/>
-      <c r="D10" s="25"/>
-      <c r="E10" s="26"/>
-      <c r="F10" s="26"/>
-      <c r="G10" s="23"/>
-      <c r="H10" s="23"/>
-      <c r="I10" s="23"/>
-      <c r="J10" s="23"/>
-      <c r="K10" s="23"/>
-      <c r="L10" s="23"/>
-      <c r="M10" s="23"/>
+      <c r="A10" s="25"/>
+      <c r="B10" s="25"/>
+      <c r="C10" s="25"/>
+      <c r="D10" s="27"/>
+      <c r="E10" s="28"/>
+      <c r="F10" s="28"/>
+      <c r="G10" s="25"/>
+      <c r="H10" s="25"/>
+      <c r="I10" s="25"/>
+      <c r="J10" s="25"/>
+      <c r="K10" s="25"/>
+      <c r="L10" s="25"/>
+      <c r="M10" s="25"/>
       <c r="N10" s="3"/>
       <c r="O10" s="3"/>
       <c r="P10" s="3"/>
@@ -1163,14 +1194,14 @@
       <c r="C11" s="11"/>
       <c r="D11" s="11"/>
       <c r="E11" s="11"/>
-      <c r="F11" s="35"/>
-      <c r="G11" s="22"/>
-      <c r="H11" s="22"/>
-      <c r="I11" s="22"/>
-      <c r="J11" s="22"/>
-      <c r="K11" s="22"/>
-      <c r="L11" s="22"/>
-      <c r="M11" s="22"/>
+      <c r="F11" s="37"/>
+      <c r="G11" s="24"/>
+      <c r="H11" s="24"/>
+      <c r="I11" s="24"/>
+      <c r="J11" s="24"/>
+      <c r="K11" s="24"/>
+      <c r="L11" s="24"/>
+      <c r="M11" s="24"/>
       <c r="N11" s="3"/>
       <c r="O11" s="3"/>
       <c r="P11" s="3"/>
@@ -1187,21 +1218,21 @@
       <c r="AA11" s="3"/>
     </row>
     <row r="12" spans="1:27" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A12" s="36" t="s">
+      <c r="A12" s="38" t="s">
         <v>23</v>
       </c>
-      <c r="B12" s="22"/>
-      <c r="C12" s="22"/>
-      <c r="D12" s="22"/>
-      <c r="E12" s="22"/>
-      <c r="F12" s="22"/>
-      <c r="G12" s="22"/>
-      <c r="H12" s="22"/>
-      <c r="I12" s="22"/>
-      <c r="J12" s="22"/>
-      <c r="K12" s="22"/>
-      <c r="L12" s="22"/>
-      <c r="M12" s="24"/>
+      <c r="B12" s="24"/>
+      <c r="C12" s="24"/>
+      <c r="D12" s="24"/>
+      <c r="E12" s="24"/>
+      <c r="F12" s="24"/>
+      <c r="G12" s="24"/>
+      <c r="H12" s="24"/>
+      <c r="I12" s="24"/>
+      <c r="J12" s="24"/>
+      <c r="K12" s="24"/>
+      <c r="L12" s="24"/>
+      <c r="M12" s="26"/>
       <c r="N12" s="3"/>
       <c r="O12" s="3"/>
       <c r="P12" s="3"/>
@@ -1227,11 +1258,11 @@
       <c r="C13" s="16" t="s">
         <v>26</v>
       </c>
-      <c r="D13" s="37" t="s">
+      <c r="D13" s="39" t="s">
         <v>27</v>
       </c>
-      <c r="E13" s="22"/>
-      <c r="F13" s="22"/>
+      <c r="E13" s="24"/>
+      <c r="F13" s="24"/>
       <c r="G13" s="17" t="s">
         <v>28</v>
       </c>
@@ -1239,7 +1270,7 @@
         <v>46226</v>
       </c>
       <c r="I13" s="14" t="s">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="J13" s="16" t="s">
         <v>29</v>
@@ -1263,21 +1294,21 @@
       <c r="AA13" s="3"/>
     </row>
     <row r="14" spans="1:27" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A14" s="36" t="s">
+      <c r="A14" s="38" t="s">
         <v>30</v>
       </c>
-      <c r="B14" s="22"/>
-      <c r="C14" s="22"/>
-      <c r="D14" s="22"/>
-      <c r="E14" s="22"/>
-      <c r="F14" s="22"/>
-      <c r="G14" s="22"/>
-      <c r="H14" s="22"/>
-      <c r="I14" s="22"/>
-      <c r="J14" s="22"/>
-      <c r="K14" s="22"/>
-      <c r="L14" s="22"/>
-      <c r="M14" s="24"/>
+      <c r="B14" s="24"/>
+      <c r="C14" s="24"/>
+      <c r="D14" s="24"/>
+      <c r="E14" s="24"/>
+      <c r="F14" s="24"/>
+      <c r="G14" s="24"/>
+      <c r="H14" s="24"/>
+      <c r="I14" s="24"/>
+      <c r="J14" s="24"/>
+      <c r="K14" s="24"/>
+      <c r="L14" s="24"/>
+      <c r="M14" s="26"/>
       <c r="N14" s="3"/>
       <c r="O14" s="3"/>
       <c r="P14" s="3"/>
@@ -1303,11 +1334,11 @@
       <c r="C15" s="16" t="s">
         <v>33</v>
       </c>
-      <c r="D15" s="37" t="s">
+      <c r="D15" s="39" t="s">
         <v>34</v>
       </c>
-      <c r="E15" s="22"/>
-      <c r="F15" s="22"/>
+      <c r="E15" s="24"/>
+      <c r="F15" s="24"/>
       <c r="G15" s="17" t="s">
         <v>35</v>
       </c>
@@ -1315,7 +1346,7 @@
         <v>46226</v>
       </c>
       <c r="I15" s="14" t="s">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="J15" s="16" t="s">
         <v>36</v>
@@ -1348,11 +1379,11 @@
       <c r="C16" s="16" t="s">
         <v>39</v>
       </c>
-      <c r="D16" s="37" t="s">
+      <c r="D16" s="39" t="s">
         <v>40</v>
       </c>
-      <c r="E16" s="22"/>
-      <c r="F16" s="22"/>
+      <c r="E16" s="24"/>
+      <c r="F16" s="24"/>
       <c r="G16" s="17" t="s">
         <v>41</v>
       </c>
@@ -1360,7 +1391,7 @@
         <v>46226</v>
       </c>
       <c r="I16" s="14" t="s">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="J16" s="16" t="s">
         <v>42</v>
@@ -1393,11 +1424,11 @@
       <c r="C17" s="16" t="s">
         <v>45</v>
       </c>
-      <c r="D17" s="37" t="s">
+      <c r="D17" s="39" t="s">
         <v>46</v>
       </c>
-      <c r="E17" s="22"/>
-      <c r="F17" s="22"/>
+      <c r="E17" s="24"/>
+      <c r="F17" s="24"/>
       <c r="G17" s="17" t="s">
         <v>47</v>
       </c>
@@ -1405,7 +1436,7 @@
         <v>46226</v>
       </c>
       <c r="I17" s="14" t="s">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="J17" s="16" t="s">
         <v>48</v>
@@ -1429,21 +1460,21 @@
       <c r="AA17" s="3"/>
     </row>
     <row r="18" spans="1:27" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A18" s="36" t="s">
+      <c r="A18" s="38" t="s">
         <v>49</v>
       </c>
-      <c r="B18" s="22"/>
-      <c r="C18" s="22"/>
-      <c r="D18" s="22"/>
-      <c r="E18" s="22"/>
-      <c r="F18" s="22"/>
-      <c r="G18" s="22"/>
-      <c r="H18" s="22"/>
-      <c r="I18" s="22"/>
-      <c r="J18" s="22"/>
-      <c r="K18" s="22"/>
-      <c r="L18" s="22"/>
-      <c r="M18" s="24"/>
+      <c r="B18" s="24"/>
+      <c r="C18" s="24"/>
+      <c r="D18" s="24"/>
+      <c r="E18" s="24"/>
+      <c r="F18" s="24"/>
+      <c r="G18" s="24"/>
+      <c r="H18" s="24"/>
+      <c r="I18" s="24"/>
+      <c r="J18" s="24"/>
+      <c r="K18" s="24"/>
+      <c r="L18" s="24"/>
+      <c r="M18" s="26"/>
       <c r="N18" s="3"/>
       <c r="O18" s="3"/>
       <c r="P18" s="3"/>
@@ -1469,11 +1500,11 @@
       <c r="C19" s="16" t="s">
         <v>52</v>
       </c>
-      <c r="D19" s="37" t="s">
+      <c r="D19" s="39" t="s">
         <v>53</v>
       </c>
-      <c r="E19" s="22"/>
-      <c r="F19" s="22"/>
+      <c r="E19" s="24"/>
+      <c r="F19" s="24"/>
       <c r="G19" s="17" t="s">
         <v>54</v>
       </c>
@@ -1481,7 +1512,7 @@
         <v>46226</v>
       </c>
       <c r="I19" s="14" t="s">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="J19" s="16" t="s">
         <v>55</v>
@@ -1514,11 +1545,11 @@
       <c r="C20" s="16" t="s">
         <v>58</v>
       </c>
-      <c r="D20" s="37" t="s">
+      <c r="D20" s="39" t="s">
         <v>59</v>
       </c>
-      <c r="E20" s="22"/>
-      <c r="F20" s="22"/>
+      <c r="E20" s="24"/>
+      <c r="F20" s="24"/>
       <c r="G20" s="17" t="s">
         <v>60</v>
       </c>
@@ -1526,7 +1557,7 @@
         <v>46226</v>
       </c>
       <c r="I20" s="14" t="s">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="J20" s="16" t="s">
         <v>55</v>
@@ -1550,21 +1581,21 @@
       <c r="AA20" s="3"/>
     </row>
     <row r="21" spans="1:27" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A21" s="36" t="s">
+      <c r="A21" s="38" t="s">
         <v>20</v>
       </c>
-      <c r="B21" s="22"/>
-      <c r="C21" s="22"/>
-      <c r="D21" s="22"/>
-      <c r="E21" s="22"/>
-      <c r="F21" s="22"/>
-      <c r="G21" s="22"/>
-      <c r="H21" s="22"/>
-      <c r="I21" s="22"/>
-      <c r="J21" s="22"/>
-      <c r="K21" s="22"/>
-      <c r="L21" s="22"/>
-      <c r="M21" s="24"/>
+      <c r="B21" s="24"/>
+      <c r="C21" s="24"/>
+      <c r="D21" s="24"/>
+      <c r="E21" s="24"/>
+      <c r="F21" s="24"/>
+      <c r="G21" s="24"/>
+      <c r="H21" s="24"/>
+      <c r="I21" s="24"/>
+      <c r="J21" s="24"/>
+      <c r="K21" s="24"/>
+      <c r="L21" s="24"/>
+      <c r="M21" s="26"/>
       <c r="N21" s="3"/>
       <c r="O21" s="3"/>
       <c r="P21" s="3"/>
@@ -1590,11 +1621,11 @@
       <c r="C22" s="16" t="s">
         <v>63</v>
       </c>
-      <c r="D22" s="37" t="s">
+      <c r="D22" s="39" t="s">
         <v>64</v>
       </c>
-      <c r="E22" s="22"/>
-      <c r="F22" s="22"/>
+      <c r="E22" s="24"/>
+      <c r="F22" s="24"/>
       <c r="G22" s="17" t="s">
         <v>65</v>
       </c>
@@ -1602,7 +1633,7 @@
         <v>46226</v>
       </c>
       <c r="I22" s="14" t="s">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="J22" s="16" t="s">
         <v>55</v>
@@ -1625,7 +1656,7 @@
       <c r="Z22" s="3"/>
       <c r="AA22" s="3"/>
     </row>
-    <row r="23" spans="1:27" ht="72.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:27" ht="111.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="14" t="s">
         <v>66</v>
       </c>
@@ -1635,11 +1666,11 @@
       <c r="C23" s="16" t="s">
         <v>68</v>
       </c>
-      <c r="D23" s="37" t="s">
+      <c r="D23" s="39" t="s">
         <v>69</v>
       </c>
-      <c r="E23" s="22"/>
-      <c r="F23" s="22"/>
+      <c r="E23" s="24"/>
+      <c r="F23" s="24"/>
       <c r="G23" s="17" t="s">
         <v>70</v>
       </c>
@@ -1647,7 +1678,7 @@
         <v>46226</v>
       </c>
       <c r="I23" s="14" t="s">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="J23" s="16" t="s">
         <v>71</v>
@@ -1656,26 +1687,28 @@
         <v>46226</v>
       </c>
       <c r="L23" s="14" t="s">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="M23" s="21" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="24" spans="1:27" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A24" s="3"/>
-      <c r="B24" s="3"/>
-      <c r="C24" s="3"/>
-      <c r="D24" s="3"/>
-      <c r="E24" s="3"/>
-      <c r="F24" s="3"/>
-      <c r="G24" s="3"/>
-      <c r="H24" s="3"/>
-      <c r="I24" s="3"/>
-      <c r="J24" s="3"/>
-      <c r="K24" s="3"/>
-      <c r="L24" s="3"/>
-      <c r="M24" s="3"/>
+      <c r="A24" s="38" t="s">
+        <v>73</v>
+      </c>
+      <c r="B24" s="24"/>
+      <c r="C24" s="24"/>
+      <c r="D24" s="24"/>
+      <c r="E24" s="24"/>
+      <c r="F24" s="24"/>
+      <c r="G24" s="24"/>
+      <c r="H24" s="24"/>
+      <c r="I24" s="24"/>
+      <c r="J24" s="24"/>
+      <c r="K24" s="24"/>
+      <c r="L24" s="24"/>
+      <c r="M24" s="26"/>
       <c r="N24" s="3"/>
       <c r="O24" s="3"/>
       <c r="P24" s="3"/>
@@ -1691,20 +1724,36 @@
       <c r="Z24" s="3"/>
       <c r="AA24" s="3"/>
     </row>
-    <row r="25" spans="1:27" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A25" s="3"/>
-      <c r="B25" s="3"/>
-      <c r="C25" s="3"/>
-      <c r="D25" s="3"/>
-      <c r="E25" s="3"/>
-      <c r="F25" s="3"/>
-      <c r="G25" s="3"/>
-      <c r="H25" s="3"/>
-      <c r="I25" s="3"/>
-      <c r="J25" s="3"/>
-      <c r="K25" s="3"/>
-      <c r="L25" s="3"/>
-      <c r="M25" s="3"/>
+    <row r="25" spans="1:27" ht="87" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="14" t="s">
+        <v>74</v>
+      </c>
+      <c r="B25" s="15" t="s">
+        <v>75</v>
+      </c>
+      <c r="C25" s="16" t="s">
+        <v>76</v>
+      </c>
+      <c r="D25" s="39" t="s">
+        <v>77</v>
+      </c>
+      <c r="E25" s="24"/>
+      <c r="F25" s="24"/>
+      <c r="G25" s="17" t="s">
+        <v>78</v>
+      </c>
+      <c r="H25" s="18">
+        <v>46252</v>
+      </c>
+      <c r="I25" s="14" t="s">
+        <v>7</v>
+      </c>
+      <c r="J25" s="16" t="s">
+        <v>79</v>
+      </c>
+      <c r="K25" s="18"/>
+      <c r="L25" s="18"/>
+      <c r="M25" s="22"/>
       <c r="N25" s="3"/>
       <c r="O25" s="3"/>
       <c r="P25" s="3"/>
@@ -1751,7 +1800,7 @@
     </row>
     <row r="27" spans="1:27" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A27" s="3"/>
-      <c r="B27" s="3"/>
+      <c r="B27" s="23"/>
       <c r="C27" s="3"/>
       <c r="D27" s="3"/>
       <c r="E27" s="3"/>
@@ -29996,22 +30045,24 @@
       <c r="AA1000" s="3"/>
     </row>
   </sheetData>
-  <mergeCells count="28">
+  <mergeCells count="30">
+    <mergeCell ref="A14:M14"/>
+    <mergeCell ref="D15:F15"/>
+    <mergeCell ref="D16:F16"/>
+    <mergeCell ref="D23:F23"/>
+    <mergeCell ref="D25:F25"/>
+    <mergeCell ref="D17:F17"/>
+    <mergeCell ref="A18:M18"/>
+    <mergeCell ref="D19:F19"/>
+    <mergeCell ref="D20:F20"/>
     <mergeCell ref="A21:M21"/>
     <mergeCell ref="D22:F22"/>
-    <mergeCell ref="D23:F23"/>
+    <mergeCell ref="A24:M24"/>
+    <mergeCell ref="L9:L10"/>
     <mergeCell ref="M9:M10"/>
     <mergeCell ref="F11:M11"/>
     <mergeCell ref="A12:M12"/>
     <mergeCell ref="D13:F13"/>
-    <mergeCell ref="A14:M14"/>
-    <mergeCell ref="D15:F15"/>
-    <mergeCell ref="D16:F16"/>
-    <mergeCell ref="L9:L10"/>
-    <mergeCell ref="D17:F17"/>
-    <mergeCell ref="A18:M18"/>
-    <mergeCell ref="D19:F19"/>
-    <mergeCell ref="D20:F20"/>
     <mergeCell ref="G9:G10"/>
     <mergeCell ref="H9:H10"/>
     <mergeCell ref="I9:I10"/>
@@ -30036,6 +30087,7 @@
     <hyperlink ref="G22" r:id="rId7" xr:uid="{00000000-0004-0000-0400-000006000000}"/>
     <hyperlink ref="G23" r:id="rId8" xr:uid="{00000000-0004-0000-0400-000007000000}"/>
     <hyperlink ref="M23" r:id="rId9" xr:uid="{00000000-0004-0000-0400-000008000000}"/>
+    <hyperlink ref="G25" r:id="rId10" xr:uid="{00000000-0004-0000-0400-000009000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>